<commit_message>
nmv 16 04 2026
</commit_message>
<xml_diff>
--- a/TS Jatai Working/Padam Input Templates/TS 1.1 Padam Input Template.xlsx
+++ b/TS Jatai Working/Padam Input Templates/TS 1.1 Padam Input Template.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ALL IMP DATA\GitHub\texts\TS Jatai Working\Padam Input Templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E5665ED-2035-46B2-810F-FADDF14528EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E765AE0F-038F-4B64-A6CC-D51943FA3813}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5704" uniqueCount="1226">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5704" uniqueCount="1227">
   <si>
     <t>PS</t>
   </si>
@@ -3786,6 +3786,9 @@
   </si>
   <si>
     <t xml:space="preserve">caqndrAgrA$H </t>
+  </si>
+  <si>
+    <t xml:space="preserve">asi# </t>
   </si>
 </sst>
 </file>
@@ -31970,8 +31973,8 @@
         <f t="shared" si="37"/>
         <v>143</v>
       </c>
-      <c r="N775" s="62" t="s">
-        <v>184</v>
+      <c r="N775" s="73" t="s">
+        <v>1226</v>
       </c>
       <c r="O775" s="8"/>
       <c r="P775" s="9"/>

</xml_diff>